<commit_message>
Added August 2026 Tournament
</commit_message>
<xml_diff>
--- a/data/source/a-town-poker-results.xlsx
+++ b/data/source/a-town-poker-results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matthewoliver/Documents/Coding/ATownPokerSite/data/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A387944-8B28-FA46-B56D-B64B972F58D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93C49593-D79C-8743-B9EE-86F9E145D19E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17480" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="38400" windowHeight="19500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="84">
   <si>
     <t>A-TOWN POKER</t>
   </si>
@@ -129,6 +129,9 @@
     <t>completed</t>
   </si>
   <si>
+    <t>upcoming</t>
+  </si>
+  <si>
     <t>TOURNAMENT RESULTS</t>
   </si>
   <si>
@@ -280,16 +283,23 @@
   </si>
   <si>
     <t>Noah S.</t>
+  </si>
+  <si>
+    <t>tournament-2026-08-01</t>
+  </si>
+  <si>
+    <t>August 2026 Tournament</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="170" formatCode="m/d/yy;@"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -580,7 +590,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -733,13 +743,9 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -761,6 +767,25 @@
     </xf>
     <xf numFmtId="166" fontId="12" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="12" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="15" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="11" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="18" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -768,6 +793,33 @@
   <dxfs count="38">
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="170" formatCode="m/d/yy;@"/>
+      <alignment horizontal="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <color rgb="FF173F32"/>
       </font>
@@ -800,30 +852,6 @@
         <scheme val="none"/>
       </font>
       <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -1264,24 +1292,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TournamentsTable" displayName="TournamentsTable" ref="A4:I6" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TournamentsTable" displayName="TournamentsTable" ref="A4:I7" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Tournament ID" dataDxfId="12"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Slug" dataDxfId="11"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Title" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Date" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Host" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Venue" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Status" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Start Time" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Initial Buy-In" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Date" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Host" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Venue" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Status" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Start Time" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Initial Buy-In" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="TournamentResultsTable" displayName="TournamentResultsTable" ref="A4:G35" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="TournamentResultsTable" displayName="TournamentResultsTable" ref="A4:G37" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:G35">
     <sortCondition ref="A6:A35"/>
   </sortState>
@@ -1595,7 +1623,7 @@
       <c r="G6" s="23"/>
       <c r="H6" s="2">
         <f>COUNTA(Tournaments!A5:A198)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="34" customHeight="1">
@@ -1613,7 +1641,7 @@
       <c r="G7" s="25"/>
       <c r="H7" s="3">
         <f>COUNTIF(Tournaments!G5:G198,"upcoming")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="34" customHeight="1">
@@ -1649,7 +1677,7 @@
       <c r="G9" s="25"/>
       <c r="H9" s="3">
         <f>COUNTA('Tournament Results'!B5:B448)+COUNTA('Cash Game Results'!B5:B461)</f>
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1738,16 +1766,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="23" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="21" style="33" customWidth="1"/>
     <col min="2" max="2" width="27" style="33" customWidth="1"/>
     <col min="3" max="3" width="34.33203125" style="33" customWidth="1"/>
-    <col min="4" max="4" width="15" style="33" customWidth="1"/>
+    <col min="4" max="4" width="15" style="69" customWidth="1"/>
     <col min="5" max="5" width="19" style="33" customWidth="1"/>
     <col min="6" max="6" width="24" style="33" customWidth="1"/>
-    <col min="7" max="8" width="13" style="33" customWidth="1"/>
+    <col min="7" max="7" width="13" style="71" customWidth="1"/>
+    <col min="8" max="8" width="13" style="33" customWidth="1"/>
     <col min="9" max="9" width="15" style="50" customWidth="1"/>
     <col min="10" max="16384" width="8.83203125" style="33"/>
   </cols>
@@ -1801,7 +1830,7 @@
       <c r="C4" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="37" t="s">
+      <c r="D4" s="67" t="s">
         <v>23</v>
       </c>
       <c r="E4" s="37" t="s">
@@ -1810,7 +1839,7 @@
       <c r="F4" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="37" t="s">
+      <c r="G4" s="52" t="s">
         <v>26</v>
       </c>
       <c r="H4" s="37" t="s">
@@ -1822,24 +1851,24 @@
     </row>
     <row r="5" spans="1:9" ht="23" customHeight="1">
       <c r="A5" s="40" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B5" s="40" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>52</v>
-      </c>
-      <c r="D5" s="54">
+        <v>53</v>
+      </c>
+      <c r="D5" s="66">
         <v>46109</v>
       </c>
       <c r="E5" s="41" t="s">
+        <v>55</v>
+      </c>
+      <c r="F5" s="41" t="s">
         <v>54</v>
       </c>
-      <c r="F5" s="41" t="s">
-        <v>53</v>
-      </c>
-      <c r="G5" s="55" t="s">
+      <c r="G5" s="54" t="s">
         <v>29</v>
       </c>
       <c r="H5" s="51"/>
@@ -1849,28 +1878,57 @@
     </row>
     <row r="6" spans="1:9" ht="23" customHeight="1">
       <c r="A6" s="47" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B6" s="47" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C6" s="48" t="s">
-        <v>72</v>
-      </c>
-      <c r="D6" s="56">
+        <v>73</v>
+      </c>
+      <c r="D6" s="68">
         <v>45913</v>
       </c>
       <c r="E6" s="48" t="s">
+        <v>55</v>
+      </c>
+      <c r="F6" s="48" t="s">
         <v>54</v>
       </c>
-      <c r="F6" s="48" t="s">
-        <v>53</v>
-      </c>
-      <c r="G6" s="55" t="s">
+      <c r="G6" s="54" t="s">
         <v>29</v>
       </c>
       <c r="H6" s="48"/>
       <c r="I6" s="49">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="23" customHeight="1">
+      <c r="A7" s="47" t="s">
+        <v>82</v>
+      </c>
+      <c r="B7" s="47" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="D7" s="68">
+        <v>46235</v>
+      </c>
+      <c r="E7" s="48" t="s">
+        <v>55</v>
+      </c>
+      <c r="F7" s="48" t="s">
+        <v>54</v>
+      </c>
+      <c r="G7" s="70" t="s">
+        <v>30</v>
+      </c>
+      <c r="H7" s="72">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="I7" s="49">
         <v>20</v>
       </c>
     </row>
@@ -1881,7 +1939,7 @@
     <mergeCell ref="A3:I3"/>
   </mergeCells>
   <conditionalFormatting sqref="G5:G198">
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="upcoming"/>
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="upcoming"/>
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation type="list" sqref="G5:G198" xr:uid="{00000000-0002-0000-0100-000000000000}">
@@ -1901,7 +1959,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="23" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="22.83203125" style="33" customWidth="1"/>
@@ -1916,7 +1974,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="23" customHeight="1">
       <c r="A1" s="32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B1" s="32"/>
       <c r="C1" s="32"/>
@@ -1927,7 +1985,7 @@
     </row>
     <row r="2" spans="1:7" ht="23" customHeight="1">
       <c r="A2" s="34" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B2" s="34"/>
       <c r="C2" s="34"/>
@@ -1952,85 +2010,85 @@
         <v>20</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C4" s="38" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D4" s="52" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E4" s="37" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F4" s="38" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G4" s="39" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="23" customHeight="1">
       <c r="A5" s="40" t="s">
-        <v>71</v>
-      </c>
-      <c r="B5" s="57" t="s">
-        <v>73</v>
-      </c>
-      <c r="C5" s="60">
+        <v>72</v>
+      </c>
+      <c r="B5" s="55" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="58">
         <v>40</v>
       </c>
-      <c r="D5" s="63" t="s">
-        <v>74</v>
-      </c>
-      <c r="E5" s="57" t="s">
-        <v>79</v>
-      </c>
-      <c r="F5" s="60">
+      <c r="D5" s="61" t="s">
+        <v>75</v>
+      </c>
+      <c r="E5" s="55" t="s">
+        <v>80</v>
+      </c>
+      <c r="F5" s="58">
         <v>100</v>
       </c>
-      <c r="G5" s="66">
+      <c r="G5" s="64">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="23" customHeight="1">
       <c r="A6" s="40" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" s="59" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6" s="57" t="s">
+        <v>76</v>
+      </c>
+      <c r="C6" s="60">
+        <v>20</v>
+      </c>
+      <c r="D6" s="63" t="s">
         <v>75</v>
       </c>
-      <c r="C6" s="62">
-        <v>20</v>
-      </c>
-      <c r="D6" s="65" t="s">
-        <v>74</v>
-      </c>
-      <c r="E6" s="59" t="s">
-        <v>79</v>
-      </c>
-      <c r="F6" s="62">
+      <c r="E6" s="57" t="s">
+        <v>80</v>
+      </c>
+      <c r="F6" s="60">
         <v>100</v>
       </c>
-      <c r="G6" s="67">
+      <c r="G6" s="65">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="23" customHeight="1">
       <c r="A7" s="40" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C7" s="50">
         <v>20</v>
       </c>
       <c r="D7" s="53" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F7" s="50">
         <v>100</v>
@@ -2041,19 +2099,19 @@
     </row>
     <row r="8" spans="1:7" ht="23" customHeight="1">
       <c r="A8" s="40" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C8" s="50">
         <v>20</v>
       </c>
       <c r="D8" s="53" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F8" s="50">
         <v>100</v>
@@ -2064,10 +2122,10 @@
     </row>
     <row r="9" spans="1:7" ht="23" customHeight="1">
       <c r="A9" s="40" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C9" s="50">
         <v>20</v>
@@ -2076,7 +2134,7 @@
         <v>5</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F9" s="50">
         <v>0</v>
@@ -2087,10 +2145,10 @@
     </row>
     <row r="10" spans="1:7" ht="23" customHeight="1">
       <c r="A10" s="40" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C10" s="50">
         <v>20</v>
@@ -2099,7 +2157,7 @@
         <v>6</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F10" s="50">
         <v>0</v>
@@ -2110,10 +2168,10 @@
     </row>
     <row r="11" spans="1:7" ht="23" customHeight="1">
       <c r="A11" s="40" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C11" s="50">
         <v>20</v>
@@ -2122,7 +2180,7 @@
         <v>7</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F11" s="50">
         <v>0</v>
@@ -2133,10 +2191,10 @@
     </row>
     <row r="12" spans="1:7" ht="23" customHeight="1">
       <c r="A12" s="40" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C12" s="50">
         <v>40</v>
@@ -2145,7 +2203,7 @@
         <v>8</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F12" s="50">
         <v>0</v>
@@ -2156,10 +2214,10 @@
     </row>
     <row r="13" spans="1:7" ht="23" customHeight="1">
       <c r="A13" s="40" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C13" s="50">
         <v>20</v>
@@ -2168,7 +2226,7 @@
         <v>9</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F13" s="50">
         <v>0</v>
@@ -2179,10 +2237,10 @@
     </row>
     <row r="14" spans="1:7" ht="23" customHeight="1">
       <c r="A14" s="40" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C14" s="50">
         <v>40</v>
@@ -2191,7 +2249,7 @@
         <v>10</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F14" s="50">
         <v>0</v>
@@ -2202,10 +2260,10 @@
     </row>
     <row r="15" spans="1:7" ht="23" customHeight="1">
       <c r="A15" s="40" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C15" s="50">
         <v>20</v>
@@ -2214,7 +2272,7 @@
         <v>11</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F15" s="50">
         <v>0</v>
@@ -2225,10 +2283,10 @@
     </row>
     <row r="16" spans="1:7" ht="23" customHeight="1">
       <c r="A16" s="40" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C16" s="50">
         <v>20</v>
@@ -2237,7 +2295,7 @@
         <v>12</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F16" s="50">
         <v>0</v>
@@ -2248,10 +2306,10 @@
     </row>
     <row r="17" spans="1:7" ht="23" customHeight="1">
       <c r="A17" s="40" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C17" s="50">
         <v>20</v>
@@ -2260,7 +2318,7 @@
         <v>13</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F17" s="50">
         <v>0</v>
@@ -2271,10 +2329,10 @@
     </row>
     <row r="18" spans="1:7" ht="23" customHeight="1">
       <c r="A18" s="40" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C18" s="50">
         <v>20</v>
@@ -2283,7 +2341,7 @@
         <v>14</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F18" s="50">
         <v>0</v>
@@ -2294,10 +2352,10 @@
     </row>
     <row r="19" spans="1:7" ht="23" customHeight="1">
       <c r="A19" s="47" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C19" s="50">
         <v>20</v>
@@ -2306,7 +2364,7 @@
         <v>15</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F19" s="50">
         <v>0</v>
@@ -2317,10 +2375,10 @@
     </row>
     <row r="20" spans="1:7" ht="23" customHeight="1">
       <c r="A20" s="47" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C20" s="50">
         <v>20</v>
@@ -2329,7 +2387,7 @@
         <v>16</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F20" s="50">
         <v>0</v>
@@ -2340,10 +2398,10 @@
     </row>
     <row r="21" spans="1:7" ht="23" customHeight="1">
       <c r="A21" s="47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" s="33" t="s">
         <v>71</v>
-      </c>
-      <c r="B21" s="33" t="s">
-        <v>70</v>
       </c>
       <c r="C21" s="50">
         <v>20</v>
@@ -2352,7 +2410,7 @@
         <v>17</v>
       </c>
       <c r="E21" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F21" s="50">
         <v>0</v>
@@ -2363,56 +2421,56 @@
     </row>
     <row r="22" spans="1:7" ht="23" customHeight="1">
       <c r="A22" s="47" t="s">
-        <v>51</v>
-      </c>
-      <c r="B22" s="58" t="s">
-        <v>55</v>
-      </c>
-      <c r="C22" s="61">
+        <v>52</v>
+      </c>
+      <c r="B22" s="56" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" s="59">
         <v>60</v>
       </c>
-      <c r="D22" s="64" t="s">
-        <v>65</v>
-      </c>
-      <c r="E22" s="58" t="s">
-        <v>38</v>
-      </c>
-      <c r="F22" s="61">
+      <c r="D22" s="62" t="s">
+        <v>66</v>
+      </c>
+      <c r="E22" s="56" t="s">
+        <v>39</v>
+      </c>
+      <c r="F22" s="59">
         <v>200</v>
       </c>
-      <c r="G22" s="61">
+      <c r="G22" s="59">
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="23" customHeight="1">
       <c r="A23" s="47" t="s">
-        <v>51</v>
-      </c>
-      <c r="B23" s="58" t="s">
-        <v>56</v>
-      </c>
-      <c r="C23" s="61">
-        <v>20</v>
-      </c>
-      <c r="D23" s="64" t="s">
-        <v>66</v>
-      </c>
-      <c r="E23" s="58" t="s">
-        <v>39</v>
-      </c>
-      <c r="F23" s="61">
+        <v>52</v>
+      </c>
+      <c r="B23" s="56" t="s">
+        <v>57</v>
+      </c>
+      <c r="C23" s="59">
+        <v>20</v>
+      </c>
+      <c r="D23" s="62" t="s">
+        <v>67</v>
+      </c>
+      <c r="E23" s="56" t="s">
+        <v>40</v>
+      </c>
+      <c r="F23" s="59">
         <v>60</v>
       </c>
-      <c r="G23" s="61">
+      <c r="G23" s="59">
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="23" customHeight="1">
       <c r="A24" s="47" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B24" s="33" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C24" s="50">
         <v>20</v>
@@ -2421,7 +2479,7 @@
         <v>3</v>
       </c>
       <c r="E24" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F24" s="50">
         <v>40</v>
@@ -2432,10 +2490,10 @@
     </row>
     <row r="25" spans="1:7" ht="23" customHeight="1">
       <c r="A25" s="47" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B25" s="33" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C25" s="50">
         <v>20</v>
@@ -2444,7 +2502,7 @@
         <v>4</v>
       </c>
       <c r="E25" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F25" s="50">
         <v>20</v>
@@ -2455,10 +2513,10 @@
     </row>
     <row r="26" spans="1:7" ht="23" customHeight="1">
       <c r="A26" s="47" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B26" s="33" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C26" s="50">
         <v>20</v>
@@ -2467,7 +2525,7 @@
         <v>5</v>
       </c>
       <c r="E26" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F26" s="50">
         <v>0</v>
@@ -2478,10 +2536,10 @@
     </row>
     <row r="27" spans="1:7" ht="23" customHeight="1">
       <c r="A27" s="47" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B27" s="33" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C27" s="50">
         <v>20</v>
@@ -2490,7 +2548,7 @@
         <v>6</v>
       </c>
       <c r="E27" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F27" s="50">
         <v>0</v>
@@ -2501,10 +2559,10 @@
     </row>
     <row r="28" spans="1:7" ht="23" customHeight="1">
       <c r="A28" s="47" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B28" s="33" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C28" s="50">
         <v>20</v>
@@ -2513,7 +2571,7 @@
         <v>7</v>
       </c>
       <c r="E28" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F28" s="50">
         <v>0</v>
@@ -2524,10 +2582,10 @@
     </row>
     <row r="29" spans="1:7" ht="23" customHeight="1">
       <c r="A29" s="47" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B29" s="33" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C29" s="50">
         <v>20</v>
@@ -2536,7 +2594,7 @@
         <v>8</v>
       </c>
       <c r="E29" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F29" s="50">
         <v>0</v>
@@ -2547,10 +2605,10 @@
     </row>
     <row r="30" spans="1:7" ht="23" customHeight="1">
       <c r="A30" s="47" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C30" s="50">
         <v>20</v>
@@ -2559,7 +2617,7 @@
         <v>9</v>
       </c>
       <c r="E30" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F30" s="50">
         <v>0</v>
@@ -2570,10 +2628,10 @@
     </row>
     <row r="31" spans="1:7" ht="23" customHeight="1">
       <c r="A31" s="47" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B31" s="33" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C31" s="50">
         <v>20</v>
@@ -2582,7 +2640,7 @@
         <v>10</v>
       </c>
       <c r="E31" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F31" s="50">
         <v>0</v>
@@ -2593,10 +2651,10 @@
     </row>
     <row r="32" spans="1:7" ht="23" customHeight="1">
       <c r="A32" s="47" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B32" s="33" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C32" s="50">
         <v>20</v>
@@ -2605,7 +2663,7 @@
         <v>11</v>
       </c>
       <c r="E32" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F32" s="50">
         <v>0</v>
@@ -2616,10 +2674,10 @@
     </row>
     <row r="33" spans="1:7" ht="23" customHeight="1">
       <c r="A33" s="47" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B33" s="33" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C33" s="50">
         <v>20</v>
@@ -2628,7 +2686,7 @@
         <v>12</v>
       </c>
       <c r="E33" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F33" s="50">
         <v>0</v>
@@ -2639,10 +2697,10 @@
     </row>
     <row r="34" spans="1:7" ht="23" customHeight="1">
       <c r="A34" s="47" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B34" s="33" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C34" s="50">
         <v>20</v>
@@ -2651,7 +2709,7 @@
         <v>13</v>
       </c>
       <c r="E34" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F34" s="50">
         <v>0</v>
@@ -2662,10 +2720,10 @@
     </row>
     <row r="35" spans="1:7" ht="23" customHeight="1">
       <c r="A35" s="47" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B35" s="33" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C35" s="50">
         <v>20</v>
@@ -2674,13 +2732,35 @@
         <v>14</v>
       </c>
       <c r="E35" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F35" s="50">
         <v>0</v>
       </c>
       <c r="G35" s="50">
         <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="23" customHeight="1">
+      <c r="A36" s="47" t="s">
+        <v>82</v>
+      </c>
+      <c r="B36" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="C36" s="50">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="23" customHeight="1">
+      <c r="A37" s="47" t="s">
+        <v>82</v>
+      </c>
+      <c r="B37" s="33" t="s">
+        <v>69</v>
+      </c>
+      <c r="C37" s="50">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -2723,7 +2803,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="34" customHeight="1">
       <c r="A1" s="29" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B1" s="29"/>
       <c r="C1" s="29"/>
@@ -2736,7 +2816,7 @@
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1">
       <c r="A2" s="30" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B2" s="30"/>
       <c r="C2" s="30"/>
@@ -2762,7 +2842,7 @@
     </row>
     <row r="4" spans="1:9" ht="34" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>21</v>
@@ -2791,28 +2871,28 @@
     </row>
     <row r="5" spans="1:9" ht="22" customHeight="1">
       <c r="A5" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D5" s="10">
         <v>46218</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G5" s="11" t="s">
         <v>29</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I5" s="9">
         <v>20</v>
@@ -2825,7 +2905,7 @@
     <mergeCell ref="A3:I3"/>
   </mergeCells>
   <conditionalFormatting sqref="G5:G199">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="upcoming"/>
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="upcoming"/>
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation type="list" sqref="G5:G199" xr:uid="{00000000-0002-0000-0300-000000000000}">
@@ -2857,7 +2937,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="21" customHeight="1">
       <c r="A1" s="32" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B1" s="32"/>
       <c r="C1" s="32"/>
@@ -2865,7 +2945,7 @@
     </row>
     <row r="2" spans="1:4" ht="21" customHeight="1">
       <c r="A2" s="34" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B2" s="34"/>
       <c r="C2" s="34"/>
@@ -2881,24 +2961,24 @@
     </row>
     <row r="4" spans="1:4" ht="21" customHeight="1">
       <c r="A4" s="36" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C4" s="38" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D4" s="39" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="21" customHeight="1">
       <c r="A5" s="40" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B5" s="41" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C5" s="42">
         <v>40</v>
@@ -2909,10 +2989,10 @@
     </row>
     <row r="6" spans="1:4" ht="21" customHeight="1">
       <c r="A6" s="40" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B6" s="44" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C6" s="45">
         <v>40</v>
@@ -2923,10 +3003,10 @@
     </row>
     <row r="7" spans="1:4" ht="21" customHeight="1">
       <c r="A7" s="40" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B7" s="44" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C7" s="45">
         <v>20</v>
@@ -2937,10 +3017,10 @@
     </row>
     <row r="8" spans="1:4" ht="21" customHeight="1">
       <c r="A8" s="40" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C8" s="45">
         <v>40</v>
@@ -2951,10 +3031,10 @@
     </row>
     <row r="9" spans="1:4" ht="21" customHeight="1">
       <c r="A9" s="40" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B9" s="44" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C9" s="45">
         <v>60</v>
@@ -2965,10 +3045,10 @@
     </row>
     <row r="10" spans="1:4" ht="21" customHeight="1">
       <c r="A10" s="40" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B10" s="44" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C10" s="45">
         <v>60</v>
@@ -2979,10 +3059,10 @@
     </row>
     <row r="11" spans="1:4" ht="21" customHeight="1">
       <c r="A11" s="47" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B11" s="48" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C11" s="49">
         <v>20</v>
@@ -2993,10 +3073,10 @@
     </row>
     <row r="12" spans="1:4" ht="21" customHeight="1">
       <c r="A12" s="47" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B12" s="48" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C12" s="49">
         <v>20</v>
@@ -3007,10 +3087,10 @@
     </row>
     <row r="13" spans="1:4" ht="21" customHeight="1">
       <c r="A13" s="47" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C13" s="50">
         <v>20</v>

</xml_diff>